<commit_message>
Cleaned up the CLI some more
</commit_message>
<xml_diff>
--- a/WorkBot/refactor/data/orders/Equal Exchange/Equal Exchange_Collegetown_2025-10-10.xlsx
+++ b/WorkBot/refactor/data/orders/Equal Exchange/Equal Exchange_Collegetown_2025-10-10.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,106 +527,52 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10400</t>
+          <t>10029</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Equal Exchange - One World</t>
+          <t>Equal Exchange - Espresso, Decaf</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>83.50</t>
+          <t>106.00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>501.00</t>
+          <t>318.00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10034</t>
+          <t>10403</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Equal Exchange - Black Silk Espresso</t>
+          <t>Equal Exchange - Cold Brew</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>77.50</t>
+          <t>83.50</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
-        <is>
-          <t>465.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>10029</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Equal Exchange - Espresso, Decaf</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>106.00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>318.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>10403</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Equal Exchange - Cold Brew</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>83.50</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
         <is>
           <t>417.50</t>
         </is>

</xml_diff>